<commit_message>
auditoria golden: registra commit no controle (d598727)
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
+++ b/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
@@ -18,9 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="10">
     <font>
       <name val="Calibri"/>
@@ -141,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -194,10 +192,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -689,14 +683,14 @@
         <v>5</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>225</v>
+        <v>158</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1879,7 +1873,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>d5ea861</t>
+          <t>recoleta-set2026</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2353,10 +2347,10 @@
         <v>30</v>
       </c>
       <c r="H36" t="n">
-        <v>647</v>
+        <v>586</v>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2370,7 +2364,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Recoleta completa set/2026 - 523+20+44+pequenas = 649 brutos; filtro Clausula 1a -&gt; 647 dentro + 2 criminais fora (14959791 matriz + 16609815 Alexandre Melchioretto); commit 22f360f</t>
+          <t>Contrato Assessoria Mensal; 1 criminal removido; sem avulsos (confissoes sem CNJ vinculado)</t>
         </is>
       </c>
     </row>
@@ -2454,11 +2448,11 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>R$ 3.242 (5 SM) + 10% exito</t>
+          <t>R$ 3.242 (5 SM)</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H38" t="n">
         <v>99</v>
@@ -2473,12 +2467,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>8cf171f</t>
+          <t>pendente</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Mensal MAQUINA DE VENDAS Franchising (1065 VIGENTE desde 01/06/2022, PDF escaneado sem OCR). 1183 e aditivo da mesma mensal. 16 empresas sem contrato proprio. Performance Franchising (675906175) movida para LSC (4a empresa contrato mensal 467); 300F passa 17-&gt;16 empresas. Nenhum avulso excluido.</t>
+          <t>Unico mensal cadastrado = Maquina de Vendas Franchising (1065). 1183 ASSINATURA = aditivo da propria mensal. Demais 16 empresas sem contrato proprio. 0 avulsos excluidos. Performance Franchising ja esta como empresa do grupo (nao duplicata).</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2492,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>8830c25cdd</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2538,41 +2532,41 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
+        <v>53</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Praiholl</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>praiholl</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>95f249611c</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2012 (id 1390244) + 1º aditivo 13/07/2026</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>R$ 7.590 (5 SM) → R$ 11.400 após aditivo</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="n">
         <v>40</v>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>BKR</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>bkr</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>7af21f27ac</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>nao migrado (sem contrato mensal no EasyJur; valor R$ 3.042,62/mes no index.html)</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>R$ 3.042,62 (SM, inicio 26/10/2020)</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>4</v>
-      </c>
-      <c r="H40" t="n">
-        <v>63</v>
-      </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2581,827 +2575,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>c24627f</t>
+          <t>93d9f84</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Sem contrato mensal no EasyJur (so 6 contratos "unico" avulsos). Exclui 2 avulsos: contrato 1692 (KRCON x Jose Biondo Filho, pasta 212/2024) e 2446 (BKR Sports x Construtora Piffer, confissao de divida de Fabio Darold Piffer).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>41</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Indusflora</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>indusflora</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>8c90de5cba</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Sem contrato mensal; 6 contratos avulsos (unico)</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>2</v>
-      </c>
-      <c r="H41" t="n">
-        <v>92</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>(a preencher)</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Sem contrato de assessoria mensal; 6 contratos avulsos (1527 BIC, 1961 Martins, 1197 Fenix, 2089/2090 ACP Zangaia, 1196 parceria). CNJs especificos nao estao na coleta atual - 0 processos a filtrar fora.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>42</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Asael</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>asael</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>9a59e6d276</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>760 (id 71343) + 1709 (id 199393 avulso)</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>R$ 5.000 (3 SM 2026)</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>6</v>
-      </c>
-      <c r="H42" t="n">
-        <v>69</v>
-      </c>
-      <c r="I42" t="n">
-        <v>10</v>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>ea2466d</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Contrato 760 "unico" migrado = assessoria mensal real (4 aditivos; 4º aditivo 27/03/2026 vig. ate 28/02/2027). Exclui 10 CNJs do contrato 1709 (Bruno Asael - ACAO 3) do original + 1 aditivo. Demais 8 contratos "unico" sao hon. sucumbenciais pontuais, nao removem processos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>43</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Cescon</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>cescon</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2429 (id 1479421) + aditivo 16/03/2026</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>R$ 7.000 + 15h/mes + 10% exito</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>12</v>
-      </c>
-      <c r="H43" t="n">
-        <v>56</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>888b8fd</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Grupo CESCON Construtora; 1º aditivo estende assessoria a 8 PJs. Vision Tower (distratada 09/2025) voltou via aditivo. Nenhum avulso.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>44</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>abc</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>17430a49f0</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Contrato PRESTACAO DE SERVICOS ADVOCATICIOS (nao migrado p/ EasyJur) - PDF em GED 8666906</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>R$ 3.992 (4 SM 2019); nao atualizado desde 2019</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>34</v>
-      </c>
-      <c r="H44" t="n">
-        <v>562</v>
-      </c>
-      <c r="I44" t="n">
-        <v>46</v>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>(a preencher)</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Contrato mensal fundador: Abelardo Benigno &amp; Costa + Embralot (2 PJs), vig. desde 15/11/2019 por 6 meses (renovado tacito). Clausula 1a par unico EXCLUI: Direito de Familia + acoes criminais de grande repercussao. Exclui 9 avulsos (contratos exito/unico 1797/2389/2384/2261/2245/1855/1819/1632/1657), 24 criminais (area 4) e 13 familia (area 1) em abas separadas. Total: 608 pos-filtro oficial, 562 DENTRO assessoria mensal (309 ativos + 253 encerrados).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>3RS</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>3rs</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>a69f8bd880</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="n">
-        <v>74</v>
-      </c>
-      <c r="I45" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>c71bcce</t>
-        </is>
-      </c>
-      <c r="L45" s="5" t="inlineStr">
-        <is>
-          <t>1 avulso removido (contrato próprio)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="7" t="n">
-        <v>42</v>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>Tajiri</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>tajiri</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>e3105a87c1</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H46" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="I46" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K46" s="7" t="inlineStr">
-        <is>
-          <t>c71bcce</t>
-        </is>
-      </c>
-      <c r="L46" s="8" t="inlineStr">
-        <is>
-          <t>1 avulso removido</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="24" customHeight="1">
-      <c r="A47" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Terra Brasil</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>terrabrasil</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>ee344ec20a</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>1085</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>R$ 7.272 (6 SM)</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="n">
-        <v>80</v>
-      </c>
-      <c r="I47" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
-          <t>c71bcce</t>
-        </is>
-      </c>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>Rhariê Robson 26 criminais contrato 2604 + Tihany 1 contrato 2566</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="7" t="n">
-        <v>44</v>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>Sunprime</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>sunprime</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>a41df437ab</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>2548</t>
-        </is>
-      </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>R$ 3.480 (IPCA)</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="H48" s="9" t="n">
-        <v>37</v>
-      </c>
-      <c r="I48" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J48" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K48" s="7" t="inlineStr">
-        <is>
-          <t>push ok sem commit extra</t>
-        </is>
-      </c>
-      <c r="L48" s="8" t="inlineStr">
-        <is>
-          <t>1 criminal fora (Cláusula Criminal exclui)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Kreibich</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>kreibich</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>1687+1476</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="n">
-        <v>93</v>
-      </c>
-      <c r="I49" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K49" s="4" t="inlineStr">
-        <is>
-          <t>merged</t>
-        </is>
-      </c>
-      <c r="L49" s="5" t="inlineStr">
-        <is>
-          <t>sem avulsos vinculados</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>5f1f58774c</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>nao (so Termo de Distrato Comercial, 2311/id 1447583)</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>sem contrato mensal cadastrado</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H50" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="I50" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
-          <t>pendente_commit</t>
-        </is>
-      </c>
-      <c r="L50" s="5" t="inlineStr">
-        <is>
-          <t>Unico contrato no EasyJur e Termo de Distrato Comercial C2 x Wagner (Baruk Res. ap. 1202), sem vinculo com os 21 processos juridicos. GED cliente so tem ConsultaOptantes. Padrao BHM/Ampempreendimentos: assessoria mensal nao digitalizada; todos DENTRO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>47</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>dvt</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>698a97d687</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>sem contrato cadastrado</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>2</v>
-      </c>
-      <c r="H51" t="n">
-        <v>21</v>
-      </c>
-      <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>e888728</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>Nenhum contrato no EasyJur; regra "sem match = DENTRO"; 0 exclusoes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>48</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Brusville</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>brusvi</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>5ab862ee28</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>1684 (id 197248)</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>R$ 6.484 (4 SM)</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>1</v>
-      </c>
-      <c r="H52" t="n">
-        <v>36</v>
-      </c>
-      <c r="I52" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Contrato tecnicamente 'unico' mas PDF confirma assessoria mensal tributaria; 0 avulsos</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="20" t="n">
-        <v>49</v>
-      </c>
-      <c r="B53" s="20" t="inlineStr">
-        <is>
-          <t>Jorcelina</t>
-        </is>
-      </c>
-      <c r="C53" s="20" t="inlineStr">
-        <is>
-          <t>jorcelina</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="inlineStr">
-        <is>
-          <t>095e4888e9</t>
-        </is>
-      </c>
-      <c r="E53" s="20" t="inlineStr">
-        <is>
-          <t>1840 (id 256227)</t>
-        </is>
-      </c>
-      <c r="F53" s="20" t="inlineStr">
-        <is>
-          <t>R$ 4.052,50 (2,5 SM 2024)</t>
-        </is>
-      </c>
-      <c r="G53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H53" s="20" t="n">
-        <v>18</v>
-      </c>
-      <c r="I53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K53" s="20" t="inlineStr">
-        <is>
-          <t>(a preencher)</t>
-        </is>
-      </c>
-      <c r="L53" s="20" t="inlineStr">
-        <is>
-          <t>Contrato ASSESSORIA MENSAL (JORCELINA DA SILVA LTDA titular) + 1o Aditivo "Jorcelina e demais" cobre as 4 PFs/PJs. Nenhum avulso. 10h tecnicas antes de hora adicional R$ 350; exito 10%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>50</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Chady</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>chady</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>4e26ecb5c2</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>1613 (id 188983)</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>R$ 4.052,50 (2,5 SM)</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>6</v>
-      </c>
-      <c r="H54" t="n">
-        <v>16</v>
-      </c>
-      <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>d4255a8 (sem alteracao)</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Sem avulsos: nenhum processo tem contrato proprio vinculado. So a PJ Chady Confeccoes tem contrato formal (1613 assessoria mensal cive/trib/trab); aditivo 2024-12-18 removeu exito trabalhista. 5 socios PF sem contrato - ficam DENTRO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>52</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Golden</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>golden</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2fbfd5c61c</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>240 (id 71204)</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>R$ 2.824 (2 SM, aditivo 2024)</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>7</v>
-      </c>
-      <c r="H55" t="n">
-        <v>31</v>
-      </c>
-      <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Assessoria mensal GRUPO GOLDEN LTDA; 5h/mes; nenhum avulso</t>
+          <t>Contrato PRAIHOLL EMPREENDIMENTOS LTDA (hoje Porto Haus); Dubai Mall PH sem contrato próprio fica DENTRO</t>
         </is>
       </c>
     </row>
@@ -3420,7 +2599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3434,7 +2613,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GRUPOS PENDENTES de auditoria filtro assessoria mensal (35 grupos)</t>
+          <t>GRUPOS PENDENTES de auditoria filtro assessoria mensal (46 grupos)</t>
         </is>
       </c>
     </row>
@@ -3483,144 +2662,144 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>abit</t>
+          <t>abc</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Grupo Abitante</t>
+          <t>Grupo ABC</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
       <c r="E5" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>brusvi</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Brusville</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>abit</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Abitante</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="9" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>gfi</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Grupo GFI</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="n">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Costa Verde</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="9" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>ads</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Grupo ADS</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>easychef</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Easychef</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>5</v>
+      <c r="F8" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>sabores</t>
+          <t>gfi</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Grupo Sabores</t>
+          <t>Grupo GFI</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>mallo</t>
+          <t>ads</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mallon</t>
+          <t>Grupo ADS</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>yany</t>
+          <t>easychef</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Grupo Yany Esquadrias de Madeira LTDA</t>
+          <t>Grupo Easychef</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr"/>
@@ -3628,547 +2807,864 @@
         <v>3</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="7" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>praiholl</t>
+          <t>sabores</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Grupo Praiholl</t>
+          <t>Grupo Sabores</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>inoven</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Inoven</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>32</v>
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>jorcelina</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Jorcelina</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>jta</t>
+          <t>asael</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Grupo JTA Empreendimentos e Urbanismo LTDA</t>
+          <t>Grupo Asael</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="7" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>rgitapema</t>
+          <t>chady</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Grupo RG Itapema Empreendimentos SPE LTDA</t>
+          <t>Grupo Chady</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr"/>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>sx</t>
+          <t>golden</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Grupo Tigipio Mineracao e Transporte de Areia e Cascalho LTDA</t>
+          <t>Grupo Golden</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>yesica</t>
+          <t>mallo</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Grupo Yesica</t>
+          <t>Grupo Mallon</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>3rs</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Grupo 3RS</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr"/>
+      <c r="E18" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>kreibich</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Kreibich</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>yany</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Yany Esquadrias de Madeira LTDA</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr"/>
+      <c r="E20" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="6" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>encoreempreendimento</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Encore Empreendimentos Imobiliarios LTDA</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="n">
+      <c r="F20" s="9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Grupo C2</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F21" s="6" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>cescon</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Cescon</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr"/>
+      <c r="E22" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>dvt</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Grupo DVT Comercio, IMPORTACAO e EXPORTACAO</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>riouruguai</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Grupo RIO Uruguai</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr"/>
-      <c r="E19" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>marcosmarceloberakha</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Marcos Marcelo Berakha</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="F23" s="6" t="n">
         <v>21</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>distribuidorapachavi</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Distribuidora Pachavi LTDA</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr"/>
-      <c r="E21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="9" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>brunaguerracarnielbl</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Bruna Guerra Carniel Blageski</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>darlandiasdacosta</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Darlan Dias da Costa</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr"/>
-      <c r="E23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>24</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>imexinvestimentosltd</t>
+          <t>indusflora</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Grupo Imex Investimentos LTDA</t>
+          <t>Grupo Indusflora Produtos Florestais S/A</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>1</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="7" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>etrzionconstrutoraei</t>
+          <t>inoven</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Grupo ETR Zion Construtora E Incorporadora LTDA</t>
+          <t>Grupo Inoven</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr"/>
       <c r="E25" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="4" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>marautopecasltda</t>
+          <t>jta</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Grupo MAR Auto Pecas LTDA</t>
+          <t>Grupo JTA Empreendimentos e Urbanismo LTDA</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F26" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>rgitapema</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Grupo RG Itapema Empreendimentos SPE LTDA</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr"/>
+      <c r="E27" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="9" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>vitalmarcomercioeind</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Vitalmar Comercio E Industria DE Pescados LTDA</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="6" t="n">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>sx</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Tigipio Mineracao e Transporte de Areia e Cascalho LTDA</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="7" t="n">
         <v>35</v>
       </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>massolindustriaecome</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Massol Industria E Comercio DE Madeiras E Transportes LTDA</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr"/>
-      <c r="E28" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>piantemodasltda</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Piante Modas LTDA</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="6" t="n">
-        <v>19</v>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>tajiri</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Itajai Comercio de Veiculos LTDA</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr"/>
+      <c r="E29" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>saolucasadministrado</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Grupo SAO Lucas Administradora DE Bens Proprios LTDA</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr"/>
-      <c r="E30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>3</v>
+      <c r="A30" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>terrabrasil</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Terra Brasil</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="4" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>estopackembalagenslt</t>
+          <t>yesica</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Grupo Estopack Embalagens LTDA</t>
+          <t>Grupo Yesica</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>encoreempreendimento</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Encore Empreendimentos Imobiliarios LTDA</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F31" s="6" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>nostraconconstrutora</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Nostracon Construtora E Incorporadora LTDA</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr"/>
-      <c r="E32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>16</v>
+      <c r="F32" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>obaobarestaurantebar</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Grupo OBA OBA Restaurante BAR LTDA</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="6" t="n">
-        <v>7</v>
+      <c r="A33" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>riouruguai</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Grupo RIO Uruguai</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
+      <c r="E33" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="7" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>jmconstrutoraeincorp</t>
+          <t>bkr</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Grupo JM Construtora E Incorporadora</t>
+          <t>Grupo BKR</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr"/>
       <c r="E34" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>marcosmarceloberakha</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Marcos Marcelo Berakha</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F34" s="9" t="n">
+      <c r="F35" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>distribuidorapachavi</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Distribuidora Pachavi LTDA</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr"/>
+      <c r="E36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>brunaguerracarnielbl</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Bruna Guerra Carniel Blageski</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>darlandiasdacosta</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Darlan Dias da Costa</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr"/>
+      <c r="E38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>imexinvestimentosltd</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Imex Investimentos LTDA</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>etrzionconstrutoraei</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Grupo ETR Zion Construtora E Incorporadora LTDA</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr"/>
+      <c r="E40" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>marautopecasltda</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Grupo MAR Auto Pecas LTDA</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>vitalmarcomercioeind</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Vitalmar Comercio E Industria DE Pescados LTDA</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>massolindustriaecome</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Massol Industria E Comercio DE Madeiras E Transportes LTDA</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr"/>
+      <c r="E43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>piantemodasltda</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Piante Modas LTDA</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>saolucasadministrado</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Grupo SAO Lucas Administradora DE Bens Proprios LTDA</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr"/>
+      <c r="E45" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>estopackembalagenslt</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Estopack Embalagens LTDA</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>nostraconconstrutora</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Nostracon Construtora E Incorporadora LTDA</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
+      <c r="E47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>obaobarestaurantebar</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Grupo OBA OBA Restaurante BAR LTDA</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1"/>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="13" t="n">
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>jmconstrutoraeincorp</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Grupo JM Construtora E Incorporadora</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr"/>
+      <c r="E49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1"/>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>Total pendentes:</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="n">
         <v>65</v>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E51" s="13" t="inlineStr">
         <is>
           <t>Procs totais pendentes:</t>
         </is>
       </c>
-      <c r="F36" s="13" t="n">
+      <c r="F51" s="13" t="n">
         <v>5292</v>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1"/>
-    <row r="38" ht="20" customHeight="1"/>
-    <row r="39" ht="20" customHeight="1"/>
-    <row r="40" ht="20" customHeight="1"/>
-    <row r="41" ht="20" customHeight="1"/>
-    <row r="42" ht="20" customHeight="1"/>
-    <row r="43" ht="20" customHeight="1"/>
-    <row r="44" ht="20" customHeight="1"/>
-    <row r="45" ht="20" customHeight="1"/>
-    <row r="46" ht="20" customHeight="1"/>
-    <row r="47" ht="20" customHeight="1"/>
-    <row r="48" ht="20" customHeight="1"/>
-    <row r="49" ht="20" customHeight="1"/>
-    <row r="50" ht="20" customHeight="1"/>
-    <row r="51" ht="20" customHeight="1"/>
     <row r="52" ht="20" customHeight="1"/>
     <row r="53" ht="20" customHeight="1"/>
     <row r="54" ht="20" customHeight="1"/>

</xml_diff>

<commit_message>
Auditoria assessoria mensal: Grupo Distribuidora Pachavi Ltda
Grupo de 1 empresa (Distribuidora Pachavi LTDA, id 679032540,
CNPJ 02.715.536/0001-19).

Contrato vigente:
- 1866 (mensal, 4 SM, R$ 5.648) - ASSESSORIA Tributario + Bancario,
  banco 14h/mes, R$450/h excedente, exito 10%. 2o Aditivo 18/06/2026
  confessa R$ 22.524 em 12x R$ 1.877 via Asaas.

Regra "sem match claro = DENTRO": todos os 18 processos permanecem
na assessoria. 9 bancarios (Bradesco/BB) + 6 tributarios (Fazenda
Nacional) + 3 civeis sem contrato avulso.

Filtros oficiais: status Ativo+Baixado+Suspenso, corte 30/09/2026.
Dashboard final: 18 processos (17 Ativo + 1 Baixado), 231,3h.

Corrige tribSub da empresa para "TJSC, TRF4, OUTROS" (igual ao panorama).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
+++ b/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="10">
     <font>
       <name val="Calibri"/>
@@ -139,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -192,6 +194,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -557,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -683,14 +689,14 @@
         <v>5</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>158</v>
+        <v>225</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1873,7 +1879,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>recoleta-set2026</t>
+          <t>d5ea861</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2347,10 +2353,10 @@
         <v>30</v>
       </c>
       <c r="H36" t="n">
-        <v>586</v>
+        <v>647</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2364,7 +2370,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Contrato Assessoria Mensal; 1 criminal removido; sem avulsos (confissoes sem CNJ vinculado)</t>
+          <t>Recoleta completa set/2026 - 523+20+44+pequenas = 649 brutos; filtro Clausula 1a -&gt; 647 dentro + 2 criminais fora (14959791 matriz + 16609815 Alexandre Melchioretto); commit 22f360f</t>
         </is>
       </c>
     </row>
@@ -2448,11 +2454,11 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>R$ 3.242 (5 SM)</t>
+          <t>R$ 3.242 (5 SM) + 10% exito</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H38" t="n">
         <v>99</v>
@@ -2467,12 +2473,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>8cf171f</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Unico mensal cadastrado = Maquina de Vendas Franchising (1065). 1183 ASSINATURA = aditivo da propria mensal. Demais 16 empresas sem contrato proprio. 0 avulsos excluidos. Performance Franchising ja esta como empresa do grupo (nao duplicata).</t>
+          <t>Mensal MAQUINA DE VENDAS Franchising (1065 VIGENTE desde 01/06/2022, PDF escaneado sem OCR). 1183 e aditivo da mesma mensal. 16 empresas sem contrato proprio. Performance Franchising (675906175) movida para LSC (4a empresa contrato mensal 467); 300F passa 17-&gt;16 empresas. Nenhum avulso excluido.</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2498,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8830c25cdd</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2532,55 +2538,1341 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
+        <v>40</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>bkr</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>7af21f27ac</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>nao migrado (sem contrato mensal no EasyJur; valor R$ 3.042,62/mes no index.html)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>R$ 3.042,62 (SM, inicio 26/10/2020)</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" t="n">
+        <v>63</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>c24627f</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Sem contrato mensal no EasyJur (so 6 contratos "unico" avulsos). Exclui 2 avulsos: contrato 1692 (KRCON x Jose Biondo Filho, pasta 212/2024) e 2446 (BKR Sports x Construtora Piffer, confissao de divida de Fabio Darold Piffer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>41</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Indusflora</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>indusflora</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>8c90de5cba</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sem contrato mensal; 6 contratos avulsos (unico)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" t="n">
+        <v>92</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>(a preencher)</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Sem contrato de assessoria mensal; 6 contratos avulsos (1527 BIC, 1961 Martins, 1197 Fenix, 2089/2090 ACP Zangaia, 1196 parceria). CNJs especificos nao estao na coleta atual - 0 processos a filtrar fora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>42</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Asael</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>asael</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>9a59e6d276</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>760 (id 71343) + 1709 (id 199393 avulso)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>R$ 5.000 (3 SM 2026)</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>6</v>
+      </c>
+      <c r="H42" t="n">
+        <v>69</v>
+      </c>
+      <c r="I42" t="n">
+        <v>10</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ea2466d</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Contrato 760 "unico" migrado = assessoria mensal real (4 aditivos; 4º aditivo 27/03/2026 vig. ate 28/02/2027). Exclui 10 CNJs do contrato 1709 (Bruno Asael - ACAO 3) do original + 1 aditivo. Demais 8 contratos "unico" sao hon. sucumbenciais pontuais, nao removem processos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>43</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cescon</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>cescon</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2429 (id 1479421) + aditivo 16/03/2026</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>R$ 7.000 + 15h/mes + 10% exito</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>12</v>
+      </c>
+      <c r="H43" t="n">
+        <v>56</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>888b8fd</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Grupo CESCON Construtora; 1º aditivo estende assessoria a 8 PJs. Vision Tower (distratada 09/2025) voltou via aditivo. Nenhum avulso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>44</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>17430a49f0</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Contrato PRESTACAO DE SERVICOS ADVOCATICIOS (nao migrado p/ EasyJur) - PDF em GED 8666906</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>R$ 3.992 (4 SM 2019); nao atualizado desde 2019</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>34</v>
+      </c>
+      <c r="H44" t="n">
+        <v>562</v>
+      </c>
+      <c r="I44" t="n">
+        <v>46</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>(a preencher)</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Contrato mensal fundador: Abelardo Benigno &amp; Costa + Embralot (2 PJs), vig. desde 15/11/2019 por 6 meses (renovado tacito). Clausula 1a par unico EXCLUI: Direito de Familia + acoes criminais de grande repercussao. Exclui 9 avulsos (contratos exito/unico 1797/2389/2384/2261/2245/1855/1819/1632/1657), 24 criminais (area 4) e 13 familia (area 1) em abas separadas. Total: 608 pos-filtro oficial, 562 DENTRO assessoria mensal (309 ativos + 253 encerrados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>3RS</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>3rs</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>a69f8bd880</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>c71bcce</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>1 avulso removido (contrato próprio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Tajiri</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>tajiri</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>e3105a87c1</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I46" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>c71bcce</t>
+        </is>
+      </c>
+      <c r="L46" s="8" t="inlineStr">
+        <is>
+          <t>1 avulso removido</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Terra Brasil</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>terrabrasil</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>ee344ec20a</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>1085</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>R$ 7.272 (6 SM)</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="I47" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>c71bcce</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Rhariê Robson 26 criminais contrato 2604 + Tihany 1 contrato 2566</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Sunprime</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>sunprime</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>a41df437ab</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>2548</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>R$ 3.480 (IPCA)</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I48" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>push ok sem commit extra</t>
+        </is>
+      </c>
+      <c r="L48" s="8" t="inlineStr">
+        <is>
+          <t>1 criminal fora (Cláusula Criminal exclui)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Kreibich</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>kreibich</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>1687+1476</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="I49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>merged</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>sem avulsos vinculados</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>5f1f58774c</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>nao (so Termo de Distrato Comercial, 2311/id 1447583)</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>sem contrato mensal cadastrado</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>pendente_commit</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Unico contrato no EasyJur e Termo de Distrato Comercial C2 x Wagner (Baruk Res. ap. 1202), sem vinculo com os 21 processos juridicos. GED cliente so tem ConsultaOptantes. Padrao BHM/Ampempreendimentos: assessoria mensal nao digitalizada; todos DENTRO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>dvt</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>698a97d687</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>sem contrato cadastrado</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>21</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>e888728</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Nenhum contrato no EasyJur; regra "sem match = DENTRO"; 0 exclusoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Brusville</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>brusvi</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>5ab862ee28</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1684 (id 197248)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>R$ 6.484 (4 SM)</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>36</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Contrato tecnicamente 'unico' mas PDF confirma assessoria mensal tributaria; 0 avulsos</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="20" t="inlineStr">
+        <is>
+          <t>Jorcelina</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>jorcelina</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>095e4888e9</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>1840 (id 256227)</t>
+        </is>
+      </c>
+      <c r="F53" s="20" t="inlineStr">
+        <is>
+          <t>R$ 4.052,50 (2,5 SM 2024)</t>
+        </is>
+      </c>
+      <c r="G53" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H53" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="I53" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K53" s="20" t="inlineStr">
+        <is>
+          <t>(a preencher)</t>
+        </is>
+      </c>
+      <c r="L53" s="20" t="inlineStr">
+        <is>
+          <t>Contrato ASSESSORIA MENSAL (JORCELINA DA SILVA LTDA titular) + 1o Aditivo "Jorcelina e demais" cobre as 4 PFs/PJs. Nenhum avulso. 10h tecnicas antes de hora adicional R$ 350; exito 10%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Chady</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>chady</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>4e26ecb5c2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1613 (id 188983)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>R$ 4.052,50 (2,5 SM)</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>6</v>
+      </c>
+      <c r="H54" t="n">
+        <v>16</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>d4255a8 (sem alteracao)</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Sem avulsos: nenhum processo tem contrato proprio vinculado. So a PJ Chady Confeccoes tem contrato formal (1613 assessoria mensal cive/trib/trab); aditivo 2024-12-18 removeu exito trabalhista. 5 socios PF sem contrato - ficam DENTRO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>golden</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2fbfd5c61c</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>240 (id 71204)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>R$ 2.824 (2 SM, aditivo 2024)</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>7</v>
+      </c>
+      <c r="H55" t="n">
+        <v>31</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Assessoria mensal GRUPO GOLDEN LTDA; 5h/mes; nenhum avulso</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Abitante</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>abit</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>c6795728b0</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>70801 / 70840 (Vera Lucia Abitante)</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>ja no HEAD</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>Sem contrato proprio excluido; regra "sem match = DENTRO". Contratos 70801 e 70840 so com PDFs escaneados; contrato 1401449 "INDENIZACAO" pode cobrir processo POSITIVA (duvida pendente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Praiholl</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>praiholl</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>83d19dcea1</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>2012 (id 1390244) + 1o Aditivo (jul/2026)</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>R$ 7.590,00 (5 SM, 18h/mes banco trimestral)</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="I57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>ja no HEAD</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>Praiholl Empreend. (hoje "Porto Haus LTDA"); 1o Aditivo 13/07/2026; Dubai Mall PH sem contrato = DENTRO. Nenhum avulso filtrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Praiholl</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>praiholl</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>95f249611c</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2012 (id 1390244) + 1º aditivo 13/07/2026</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>R$ 7.590 (5 SM) → R$ 11.400 após aditivo</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Mallon</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>mallo</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>309fc6537d</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>1669 (id 195709)</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>R$ 3.242,00 (2 SM)</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="I58" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H40" t="n">
-        <v>40</v>
-      </c>
-      <c r="I40" t="n">
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>ja no HEAD (d4255a8)</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="inlineStr">
+        <is>
+          <t>Exclui 2 avulsos contrato 2137 Registro de Marca (CNJs 940140349/940161214, Felipe Mallon via NOMA id 682374145). Mensal 1669 Mallon Empreend. 2 SM + exito 10% + R$500/h excedente. Contratos extrajudiciais 1647/2367/2200/2019 sem CNJ no painel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>54</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Distribuidora Pachavi</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>distribuidorapachavi</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>47d02ea071</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>1866 (id 258350)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>R$ 5.648,00 (4 SM, 14h/mes)</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>18</v>
+      </c>
+      <c r="H59" t="n">
         <v>0</v>
       </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>93d9f84</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Contrato PRAIHOLL EMPREENDIMENTOS LTDA (hoje Porto Haus); Dubai Mall PH sem contrato próprio fica DENTRO</t>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>pendente push</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Mensal 4 SM Tributario+Bancario, banco 14h/mes, R$450/h excedente. 2o Aditivo 18/06/2026 confessa R$22.524 em 12x R$1.877. Todos 18 procs DENTRO: 9 bancarios + 6 tributarios + 3 civeis sem match claro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>55</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Massol</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>massolindustriaecome</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1cc21963cd</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2144 (id 1411231)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>R$ 4.863 (3 SM)</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" t="n">
+        <v>15</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Mensal 3 SM Tributario+Bancario (BB/Bradesco/Sicoob), exito 8%. Todos 15 procs DENTRO: 7 tributarios + 7 bancarios + 1 civel (Butzke, sem match claro = DENTRO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>56</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Piante Modas Ltda</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>piantemodasltda</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>054983cdcb</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>1858 (id 257696)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>R$ 3.242,00 (2,5 SM)</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="n">
+        <v>20</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Mensal 1858 ASSESSORIA MENSAL banc e RJ (2,5 SM); aditivo 2025-07-08 (3,25 SM depois 3 SM). Contrato avulso 2555 REVISAO TRIBUTARIA R$ 25.000 e pedido administrativo TTD/SEFAZ-SC, sem CNJ vinculado. Todos 20 procs DENTRO (16 Ativo + 4 Baixado): 19 bancario + 1 recuperacao judicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Tigipio Mineração</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>sx</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>f155d076a5</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>1799 (id 211483)</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>R$ 8.105 (5,34 SM)</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H62" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="I62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>pendente push</t>
+        </is>
+      </c>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>Contrato único 1799 (ASSESSORIA MENSAL VIGENTE desde 06/08/2024) na Tigipio Mineração; demais 5 empresas (SX Transporte, SX Argila, Andre/Sandra/Gabriela Schütz) sem contrato próprio no EasyJur. Nenhum avulso identificado (todos processos têm contrato=null). 42 procs DENTRO após filtros oficiais (status Ativo/Baixado/Suspenso + corte 2026-09-30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>58</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Estopack Embalagens</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>estopackembalagenslt</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>5b992a1ed6</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>1843 (id 256446)</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>R$ 4.000,00 (2,833 SM 2024)</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="n">
+        <v>17</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Darlan Dias da Costa</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>darlandiasdacosta</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>e0a39aef44</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>1083 (id 125279)</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>R$ 2.431,50 (1,5 SM)</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="I64" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Mensal 1083 ASSESSORIA MENSAL 1,5 SM (apos 6m iniciais a 1 SM) + 10% exito. Objeto: Consultivo + Contratos + Contencioso civel/trabalhista. 2 avulsos vigentes excluidos: 2138 (medida protetiva CNJ 5006761-30.2025.8.24.0005, R$ 25k) e 2139 (dissolucao uniao estavel + partilha + guarda, pasta 169/2025, R$ 12,5k). Alimentos (5008095/2025 e 5013845/2026) permanecem DENTRO (objeto do 2139 nao cobre alimentos).</t>
         </is>
       </c>
     </row>
@@ -2599,7 +3891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2613,7 +3905,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GRUPOS PENDENTES de auditoria filtro assessoria mensal (46 grupos)</t>
+          <t>GRUPOS PENDENTES de auditoria filtro assessoria mensal (23 grupos)</t>
         </is>
       </c>
     </row>
@@ -2662,20 +3954,20 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>gfi</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Grupo ABC</t>
+          <t>Grupo GFI</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
       <c r="E5" s="7" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>615</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -2684,20 +3976,20 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>brusvi</t>
+          <t>ads</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Grupo Brusville</t>
+          <t>Grupo ADS</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -2706,42 +3998,42 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>abit</t>
+          <t>easychef</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Grupo Abitante</t>
+          <t>Grupo Easychef</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Costa Verde</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>38</v>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>sabores</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Sabores</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -2750,276 +4042,276 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>gfi</t>
+          <t>yany</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Grupo GFI</t>
+          <t>Grupo Yany Esquadrias de Madeira LTDA</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>inoven</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Inoven</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="9" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>ads</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Grupo ADS</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="9" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>jta</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Grupo JTA Empreendimentos e Urbanismo LTDA</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>easychef</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Easychef</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="9" t="n">
-        <v>5</v>
+      <c r="F11" s="6" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>sabores</t>
+          <t>rgitapema</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Grupo Sabores</t>
+          <t>Grupo RG Itapema Empreendimentos SPE LTDA</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="9" t="n">
         <v>3</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>jorcelina</t>
+          <t>yesica</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Grupo Jorcelina</t>
+          <t>Grupo Yesica</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>asael</t>
+          <t>encoreempreendimento</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Grupo Asael</t>
+          <t>Grupo Encore Empreendimentos Imobiliarios LTDA</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>81</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>chady</t>
+          <t>riouruguai</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Grupo Chady</t>
+          <t>Grupo RIO Uruguai</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr"/>
       <c r="E15" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>golden</t>
+          <t>marcosmarceloberakha</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Grupo Golden</t>
+          <t>Grupo Marcos Marcelo Berakha</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>mallo</t>
+          <t>brunaguerracarnielbl</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mallon</t>
+          <t>Grupo Bruna Guerra Carniel Blageski</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>imexinvestimentosltd</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Imex Investimentos LTDA</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>3rs</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Grupo 3RS</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr"/>
-      <c r="E18" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="n">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>etrzionconstrutoraei</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Grupo ETR Zion Construtora E Incorporadora LTDA</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
+      <c r="E19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>kreibich</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Kreibich</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>yany</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Yany Esquadrias de Madeira LTDA</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr"/>
-      <c r="E20" s="7" t="n">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>marautopecasltda</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Grupo MAR Auto Pecas LTDA</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>c2</t>
+          <t>vitalmarcomercioeind</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Grupo C2</t>
+          <t>Grupo Vitalmar Comercio E Industria DE Pescados LTDA</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr"/>
@@ -3027,644 +4319,123 @@
         <v>1</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="7" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>cescon</t>
+          <t>saolucasadministrado</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Grupo Cescon</t>
+          <t>Grupo SAO Lucas Administradora DE Bens Proprios LTDA</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr"/>
       <c r="E22" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>dvt</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Grupo DVT Comercio, IMPORTACAO e EXPORTACAO</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>21</v>
+      <c r="A23" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>nostraconconstrutora</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Nostracon Construtora E Incorporadora LTDA</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr"/>
+      <c r="E23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>indusflora</t>
+          <t>obaobarestaurantebar</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Grupo Indusflora Produtos Florestais S/A</t>
+          <t>Grupo OBA OBA Restaurante BAR LTDA</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>93</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="7" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>inoven</t>
+          <t>jmconstrutoraeincorp</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Grupo Inoven</t>
+          <t>Grupo JM Construtora E Incorporadora</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr"/>
       <c r="E25" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>jta</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Grupo JTA Empreendimentos e Urbanismo LTDA</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>rgitapema</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Grupo RG Itapema Empreendimentos SPE LTDA</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr"/>
-      <c r="E27" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>sx</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Tigipio Mineracao e Transporte de Areia e Cascalho LTDA</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F28" s="6" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>tajiri</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Itajai Comercio de Veiculos LTDA</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr"/>
-      <c r="E29" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>terrabrasil</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Terra Brasil</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F30" s="6" t="n">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>yesica</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Yesica</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F31" s="6" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>encoreempreendimento</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Encore Empreendimentos Imobiliarios LTDA</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="7" t="n">
-        <v>41</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>riouruguai</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Grupo RIO Uruguai</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr"/>
-      <c r="E33" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F33" s="9" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>bkr</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Grupo BKR</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr"/>
-      <c r="E34" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F34" s="9" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>marcosmarceloberakha</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Marcos Marcelo Berakha</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>distribuidorapachavi</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Distribuidora Pachavi LTDA</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr"/>
-      <c r="E36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="9" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>brunaguerracarnielbl</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Bruna Guerra Carniel Blageski</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="7" t="n">
-        <v>47</v>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>darlandiasdacosta</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Darlan Dias da Costa</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr"/>
-      <c r="E38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>imexinvestimentosltd</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Imex Investimentos LTDA</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="7" t="n">
-        <v>49</v>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>etrzionconstrutoraei</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>Grupo ETR Zion Construtora E Incorporadora LTDA</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr"/>
-      <c r="E40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>marautopecasltda</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Grupo MAR Auto Pecas LTDA</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>vitalmarcomercioeind</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Vitalmar Comercio E Industria DE Pescados LTDA</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="6" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="7" t="n">
-        <v>53</v>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>massolindustriaecome</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Massol Industria E Comercio DE Madeiras E Transportes LTDA</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr"/>
-      <c r="E43" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="9" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>piantemodasltda</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Piante Modas LTDA</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="6" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>saolucasadministrado</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Grupo SAO Lucas Administradora DE Bens Proprios LTDA</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr"/>
-      <c r="E45" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>estopackembalagenslt</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Estopack Embalagens LTDA</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="6" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="7" t="n">
-        <v>57</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>nostraconconstrutora</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Nostracon Construtora E Incorporadora LTDA</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr"/>
-      <c r="E47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="9" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>obaobarestaurantebar</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Grupo OBA OBA Restaurante BAR LTDA</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="6" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="7" t="n">
-        <v>59</v>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>jmconstrutoraeincorp</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>Grupo JM Construtora E Incorporadora</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr"/>
-      <c r="E49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="9" t="n">
-        <v>7</v>
-      </c>
-    </row>
+    <row r="26" ht="20" customHeight="1"/>
+    <row r="27" ht="20" customHeight="1"/>
+    <row r="28" ht="20" customHeight="1"/>
+    <row r="29" ht="20" customHeight="1"/>
+    <row r="30" ht="20" customHeight="1"/>
+    <row r="31" ht="20" customHeight="1"/>
+    <row r="32" ht="20" customHeight="1"/>
+    <row r="33" ht="20" customHeight="1"/>
+    <row r="34" ht="20" customHeight="1"/>
+    <row r="35" ht="20" customHeight="1"/>
+    <row r="36" ht="20" customHeight="1"/>
+    <row r="37" ht="20" customHeight="1"/>
+    <row r="38" ht="20" customHeight="1"/>
+    <row r="39" ht="20" customHeight="1"/>
+    <row r="40" ht="20" customHeight="1"/>
+    <row r="41" ht="20" customHeight="1"/>
+    <row r="42" ht="20" customHeight="1"/>
+    <row r="43" ht="20" customHeight="1"/>
+    <row r="44" ht="20" customHeight="1"/>
+    <row r="45" ht="20" customHeight="1"/>
+    <row r="46" ht="20" customHeight="1"/>
+    <row r="47" ht="20" customHeight="1"/>
+    <row r="48" ht="20" customHeight="1"/>
+    <row r="49" ht="20" customHeight="1"/>
     <row r="50" ht="20" customHeight="1"/>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>Total pendentes:</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="n">
-        <v>65</v>
-      </c>
-      <c r="E51" s="13" t="inlineStr">
-        <is>
-          <t>Procs totais pendentes:</t>
-        </is>
-      </c>
-      <c r="F51" s="13" t="n">
-        <v>5292</v>
-      </c>
-    </row>
+    <row r="51" ht="20" customHeight="1"/>
     <row r="52" ht="20" customHeight="1"/>
     <row r="53" ht="20" customHeight="1"/>
     <row r="54" ht="20" customHeight="1"/>

</xml_diff>

<commit_message>
auditoria sx: registra commit no controle (5fa8111)
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
+++ b/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
@@ -594,6 +594,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3720,7 +3721,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>ja no HEAD (8b61aca)</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -3774,7 +3775,7 @@
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
-          <t>pendente push</t>
+          <t>5fa8111</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
@@ -3882,34 +3883,34 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Inoven</t>
+          <t>Marcos Marcelo Berakha</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>inoven</t>
+          <t>marcosmarceloberakha</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>7db7a2600e</t>
+          <t>05b2369b17</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1140 (id 132415)</t>
+          <t>2104 (id 1407493) HONORARIOS/unico</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>R$ 4.554 (3 SM / 8h banco semestral - aditivo 22/04/2025)</t>
+          <t>R$ 6.484,00 (12x R$ 10.000 + 12,5% exito)</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H65" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="I65" t="n">
         <v>0</v>
@@ -3921,12 +3922,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Contrato original era por ato (licitacoes); 1 Aditivo (22/04/2025) migrou para assessoria mensal. Empresa 681546826 sem contrato proprio mas mesmo CNPJ raiz. 0 avulsos.</t>
+          <t>Contrato 2104 ESPECIFICO para "sete acoes judiciais" indicadas via parceria com Jorge Antonio Maurique Soc. Ind. Advocacia (50% repasse pro-labore/exito). Classificacao UNICO (nao mensal). PDF principal (file_id 7608153) escaneado. Nenhum processo com id_contrato associado; REGRA CRAVADA aplicada = todos DENTRO. 20 procs apos corte 30/09 (2 cadastros em outubro ficam fora deste corte).</t>
         </is>
       </c>
     </row>
@@ -3970,7 +3971,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4114,69 +4114,69 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>inoven</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Grupo Inoven</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>jta</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Grupo JTA Empreendimentos e Urbanismo LTDA</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="n">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F11" s="6" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>rgitapema</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Grupo RG Itapema Empreendimentos SPE LTDA</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="n">
+      <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F12" s="9" t="n">
         <v>3</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>yesica</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Yesica</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -4185,69 +4185,69 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>encoreempreendimento</t>
+          <t>yesica</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Grupo Encore Empreendimentos Imobiliarios LTDA</t>
+          <t>Grupo Yesica</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>encoreempreendimento</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Encore Empreendimentos Imobiliarios LTDA</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F14" s="6" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>riouruguai</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Grupo RIO Uruguai</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr"/>
-      <c r="E14" s="7" t="n">
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F15" s="9" t="n">
         <v>4</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>marcosmarceloberakha</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Marcos Marcelo Berakha</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -4269,7 +4269,7 @@
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
@@ -4313,7 +4313,7 @@
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -4335,7 +4335,7 @@
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
@@ -4357,7 +4357,7 @@
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
@@ -4379,7 +4379,7 @@
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auditoria contratos Grupo Inoven: 32 processos dentro, 0 avulsos fora
Grupo com 2 empresas (Inoven Comercio Internacional id 2129803 e
Inoven Industria Comercio Importacao id 681546826, mesmo CNPJ raiz).

Unico contrato cadastrado no EasyJur: 1140 (id 132415).
- Original 03/11/2022: por ato (licitacoes), 0,5-3 SM por licitacao + 5% exito.
- 1 Aditivo 22/04/2025 (lido na integra, GED 7679878): MIGRA para assessoria
  mensal - 3 SM/mes (R$ 4.554), 8h tecnicas/mes com banco semestral,
  hora excedente R$ 500, prazo indeterminado.

Nenhum processo com contrato_id vinculado; sem CNJ identificado nos PDFs
para exclusao. 0 processos avulsos fora do painel.

Alteracoes:
- index.html + c/7db7a2600e/index.html: inoven em _CORTE_POR_GRUPO (30/09/2026).
- PLANILHA_MESTRE_INOVEN.xlsx: nova.
- CONTROLE_AUDITORIA_ASSESSORIA.xlsx: inoven movida de Pendentes para
  Grupos auditados (ficam 20 pendentes).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
+++ b/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3931,6 +3931,60 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Vitalmar</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>vitalmarcomercioeind</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>433f78499e</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>nao mensal (contratos avulsos 1411237 e 1437681 HONORARIOS/unico)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Sem assessoria mensal - contratos avulsos (4 SM exito 10/20% + 1 SM exito 25%)</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" t="n">
+        <v>35</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Cliente SEM contrato de assessoria mensal cadastrado no EasyJur. 2 contratos VIGENTE HONORARIOS/unico (1411237 4SM 4 bancos exito 10/20%; 1437681 1SM exito 25%). PDFs sao escaneados, mas observacoes do EasyJur dao escopo generico (sem CNJ). Nenhum processo com contrato_id nos brutos. 0 exclusoes, todos 35 processos DENTRO.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
@@ -3946,7 +4000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3971,6 +4025,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4334,39 +4389,39 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>vitalmarcomercioeind</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Vitalmar Comercio E Industria DE Pescados LTDA</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="n">
+      <c r="A20" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>saolucasadministrado</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Grupo SAO Lucas Administradora DE Bens Proprios LTDA</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr"/>
+      <c r="E20" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="6" t="n">
-        <v>35</v>
+      <c r="F20" s="9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>saolucasadministrado</t>
+          <t>nostraconconstrutora</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Grupo SAO Lucas Administradora DE Bens Proprios LTDA</t>
+          <t>Grupo Nostracon Construtora E Incorporadora LTDA</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr"/>
@@ -4374,75 +4429,54 @@
         <v>1</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>nostraconconstrutora</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Grupo Nostracon Construtora E Incorporadora LTDA</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr"/>
-      <c r="E22" s="7" t="n">
+      <c r="A22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>obaobarestaurantebar</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Grupo OBA OBA Restaurante BAR LTDA</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="9" t="n">
-        <v>16</v>
+      <c r="F22" s="6" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>obaobarestaurantebar</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Grupo OBA OBA Restaurante BAR LTDA</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="n">
+      <c r="A23" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>jmconstrutoraeincorp</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Grupo JM Construtora E Incorporadora</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr"/>
+      <c r="E23" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F23" s="9" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>jmconstrutoraeincorp</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Grupo JM Construtora E Incorporadora</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr"/>
-      <c r="E24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>7</v>
-      </c>
-    </row>
+    <row r="24" ht="20" customHeight="1"/>
     <row r="25" ht="20" customHeight="1"/>
     <row r="26" ht="20" customHeight="1"/>
     <row r="27" ht="20" customHeight="1"/>

</xml_diff>

<commit_message>
auditoria vitalmar: registra commit no controle (245e83c)
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
+++ b/CONTROLE_AUDITORIA_ASSESSORIA.xlsx
@@ -594,6 +594,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3975,7 +3976,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>HEAD</t>
+          <t>245e83c</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -4024,7 +4025,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>